<commit_message>
DATA. Entrenamiento que faltaba de modelos en USA y ENG + assess
</commit_message>
<xml_diff>
--- a/data/usa/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/usa/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,45 +507,45 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>A3m1Vera</t>
+          <t>CAvUgWQG</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45549.85416666666</v>
+        <v>45556.625</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">villarreal a 
+          <t xml:space="preserve">freemon j 
   usa </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mercedes benz stadium
-  atlanta  ga </t>
+          <t xml:space="preserve">yankee stadium
+  new york  ny </t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>71000</v>
+        <v>54251</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>EPngUvhk</t>
+          <t>vZraQYnO</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>atlanta utd</t>
+          <t>new york city</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>84yIDQMe</t>
+          <t>0AheRyBg</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>nashville sc</t>
+          <t>inter miami</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -574,45 +574,45 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>8lOY3V6E</t>
+          <t>6XwYhjtN</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45549.85416666666</v>
+        <v>45556.70833333334</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">vazquez r 
+          <t xml:space="preserve">allatin m 
   usa </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">saputo stadium
-  montreal  qc </t>
+          <t xml:space="preserve">bank of america stadium
+  charlotte  nc </t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>23112</v>
+        <v>74867</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>j9cigLCr</t>
+          <t>QJF7WTFB</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>cf montreal</t>
+          <t>charlotte</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>QJF7WTFB</t>
+          <t>tr3oe8I8</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>charlotte</t>
+          <t>new england revolution</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -641,45 +641,45 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>ITj9TZCB</t>
+          <t>rBhIe7Ef</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45549.85416666666</v>
+        <v>45556.85416666666</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">touchan r 
+          <t xml:space="preserve">szpala l 
   usa </t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">audi field
-  washington  dc </t>
+          <t xml:space="preserve">saputo stadium
+  montreal  qc </t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>20000</v>
+        <v>23112</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>O6hjfSXE</t>
+          <t>j9cigLCr</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>dc united</t>
+          <t>cf montreal</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>vZraQYnO</t>
+          <t>UwAwNo2E</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>new york city</t>
+          <t>chicago fire</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -708,45 +708,45 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>lfn5UFc5</t>
+          <t>I7sxhAeT</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45549.85416666666</v>
+        <v>45556.85416666666</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">dickerson j 
-  usa </t>
+          <t xml:space="preserve">boiko s 
+  ukr </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">tql stadium
-  cincinnati  oh </t>
+          <t xml:space="preserve">lower com field
+  columbus  oh </t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26000</v>
+        <v>20371</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>8btog05R</t>
+          <t>pQ8rarA7</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>fc cincinnati</t>
+          <t>columbus crew</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>pQ8rarA7</t>
+          <t>rsHkUNCo</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>columbus crew</t>
+          <t>orlando city</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -775,45 +775,45 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>dKkDSgSH</t>
+          <t>OlK4mU3p</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45549.85416666666</v>
+        <v>45556.85416666666</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">boiko s 
-  ukr </t>
+          <t xml:space="preserve">penso c 
+  usa </t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">chase stadium
-  fort lauderdale  fl </t>
+          <t xml:space="preserve">red bull arena
+  harrison  nj </t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>21550</v>
+        <v>25000</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0AheRyBg</t>
+          <t>zV5YmQAr</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>inter miami</t>
+          <t>new york red bulls</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Szrwix67</t>
+          <t>EPngUvhk</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>philadelphia union</t>
+          <t>atlanta utd</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -842,45 +842,45 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>vquIRDsO</t>
+          <t>2uJ8nlJj</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45549.85416666666</v>
+        <v>45556.89583333334</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">penso t 
+          <t xml:space="preserve">rivas v 
   usa </t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">inter co stadium
-  orlando  fl </t>
+          <t xml:space="preserve">q2 stadium
+  austin  tx </t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>25500</v>
+        <v>20738</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>rsHkUNCo</t>
+          <t>IeT6JBE3</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>orlando city</t>
+          <t>austin fc</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>tr3oe8I8</t>
+          <t>2i4sdl32</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>new england revolution</t>
+          <t>houston dynamo</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -909,45 +909,45 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>jDDw3kMK</t>
+          <t>jeCjBXei</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45549.85416666666</v>
+        <v>45556.89583333334</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">penso c 
+          <t xml:space="preserve">da silva a 
   usa </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">bmo field
-  toronto  on </t>
+          <t xml:space="preserve">toyota stadium
+  frisco  tx </t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>30991</v>
+        <v>20500</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>zsdfgnmL</t>
+          <t>4GtbI4Q1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>toronto fc</t>
+          <t>fc dallas</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>IeT6JBE3</t>
+          <t>txUJt9AR</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>austin fc</t>
+          <t>los angeles fc</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -976,45 +976,45 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>xUcLQXdU</t>
+          <t>CA0a9BQ3</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45549.89583333334</v>
+        <v>45556.89583333334</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">allatin m 
-  usa </t>
+          <t xml:space="preserve">lauziere p 
+  can </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">soldier field
-  chicago  il </t>
+          <t xml:space="preserve">geodis park
+  nashville  tn </t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>61500</v>
+        <v>30000</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>UwAwNo2E</t>
+          <t>84yIDQMe</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>chicago fire</t>
+          <t>nashville sc</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>zV5YmQAr</t>
+          <t>8btog05R</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>new york red bulls</t>
+          <t>fc cincinnati</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -1043,45 +1043,45 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>EkZQoHSu</t>
+          <t>UoBfAiBc</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45549.89583333334</v>
+        <v>45556.89583333334</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">freemon j 
+          <t xml:space="preserve">pekmic i 
   usa </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">shell energy stadium
-  houston  tx </t>
+          <t xml:space="preserve">children s mercy park
+  kansas city  ks </t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>22039</v>
+        <v>21650</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2i4sdl32</t>
+          <t>CURGfJWt</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>houston dynamo</t>
+          <t>sporting kansas city</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>W0ealpQl</t>
+          <t>zXFxsw2a</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>real salt lake</t>
+          <t>minnesota united</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -1110,45 +1110,45 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>htYUpyrn</t>
+          <t>tdBLfRT0</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45549.89583333334</v>
+        <v>45556.9375</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">de oliveira m 
+          <t xml:space="preserve">mendoza r 
   usa </t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">citypark
-  st  louis  mo </t>
+          <t xml:space="preserve">dick s sporting goods park
+  commerce city  co </t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>22423</v>
+        <v>18061</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>4r4sKQud</t>
+          <t>jmBZNRn8</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>st  louis city</t>
+          <t>colorado rapids</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>zXFxsw2a</t>
+          <t>zsdfgnmL</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>minnesota united</t>
+          <t>toronto fc</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1177,35 +1177,35 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>AHSZqech</t>
+          <t>QD438VuA</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45549.9375</v>
+        <v>45556.9375</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">dujic f 
-  can </t>
+          <t xml:space="preserve">penso t 
+  usa </t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">dick s sporting goods park
-  commerce city  co </t>
+          <t xml:space="preserve">america first field
+  sandy  ut </t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>18061</v>
+        <v>20213</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>jmBZNRn8</t>
+          <t>W0ealpQl</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>colorado rapids</t>
+          <t>real salt lake</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1244,15 +1244,15 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>l8RwqFCb</t>
+          <t>zJAPgoq7</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45549.97916666666</v>
+        <v>45556.97916666666</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">unkel t 
+          <t xml:space="preserve">marrufo j 
   usa </t>
         </is>
       </c>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>txUJt9AR</t>
+          <t>K2dlua5N</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>los angeles fc</t>
+          <t>vancouver whitecaps</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1311,45 +1311,45 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>foKU4Bi8</t>
+          <t>Kz477keG</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45549.97916666666</v>
+        <v>45556.97916666666</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">szpala l 
-  usa </t>
+          <t xml:space="preserve">montero r 
+  cos </t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">bc place
-  vancouver  bc </t>
+          <t xml:space="preserve">paypal park
+  san jose  ca </t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>54405</v>
+        <v>18000</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>K2dlua5N</t>
+          <t>x05z14ue</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>vancouver whitecaps</t>
+          <t>san jose earthquakes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>x05z14ue</t>
+          <t>4r4sKQud</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>san jose earthquakes</t>
+          <t>st  louis city</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1370,73 +1370,6 @@
         </is>
       </c>
       <c r="O14" t="inlineStr">
-        <is>
-          <t>mls</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>rVQsrZR4</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>45550.84375</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fischer d 
-  can </t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">lumen field
-  seattle  wa </t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>72000</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>6P5S63Ah</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>seattle sounders</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>CURGfJWt</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>sporting kansas city</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>167</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1671</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>2024</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>usa</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
         <is>
           <t>mls</t>
         </is>

</xml_diff>